<commit_message>
docs: Agregados Story Points iniciales, se hará merge hasta conocer el puntaje que se indique como puntaje final
</commit_message>
<xml_diff>
--- a/Documentacion/1. Story_Points_y_Asignacion_de_Responsabilidades.xlsx
+++ b/Documentacion/1. Story_Points_y_Asignacion_de_Responsabilidades.xlsx
@@ -86,7 +86,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
   <si>
     <t xml:space="preserve">Integrantes Proyecto</t>
   </si>
@@ -223,7 +223,7 @@
     <t>MAT1</t>
   </si>
   <si>
-    <t xml:space="preserve">Servicio para Administrar Pre-Matrícula</t>
+    <t xml:space="preserve">Servicio para Administrar Prematrícula</t>
   </si>
   <si>
     <t>MAT2</t>
@@ -304,75 +304,147 @@
     <t>ADM1</t>
   </si>
   <si>
+    <t xml:space="preserve">Plantilla Web </t>
+  </si>
+  <si>
     <t>ADM2</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Login</t>
+  </si>
+  <si>
     <t>ADM3</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web de Bienvenida</t>
+  </si>
+  <si>
     <t>ADM4</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Usuarios</t>
+  </si>
+  <si>
     <t>ADM5</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Roles</t>
+  </si>
+  <si>
     <t>ADM6</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Parametros</t>
+  </si>
+  <si>
     <t>ADM7</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Módulos</t>
+  </si>
+  <si>
     <t>ADM8</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Instituciones</t>
+  </si>
+  <si>
     <t>ADM9</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Carreas</t>
+  </si>
+  <si>
     <t>ADM10</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Cursos</t>
+  </si>
+  <si>
     <t>ADM11</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Profesores</t>
+  </si>
+  <si>
     <t>ADM12</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Periodos</t>
+  </si>
+  <si>
     <t>ADM13</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Grupos</t>
+  </si>
+  <si>
     <t>ADM14</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Prematrículas</t>
+  </si>
+  <si>
     <t>ADM15</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Matrículas</t>
+  </si>
+  <si>
     <t>ADM16</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Expedientes</t>
+  </si>
+  <si>
     <t>ADM17</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Cargar Desgloses y Asignar/Modificar Notas</t>
+  </si>
+  <si>
     <t>ADM18</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Visualizar Promedios</t>
+  </si>
+  <si>
     <t>ADM19</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Obtener Listados de Estudianters</t>
+  </si>
+  <si>
     <t>ADM20</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Web para Administrar Facturas</t>
+  </si>
+  <si>
     <t>ADM21</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla para Administrar Pagos</t>
+  </si>
+  <si>
     <t>ADM22</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla para Enviar Notificaciones por Correo</t>
+  </si>
+  <si>
     <t>ADM23</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla para Consultar Bitácora</t>
+  </si>
+  <si>
     <t>ADM24</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla para Ver Perfil y Cambiar Contraseña</t>
+  </si>
+  <si>
     <t xml:space="preserve">Historia de Usuario (Tercer Sprint)</t>
   </si>
   <si>
@@ -382,31 +454,58 @@
     <t>MOB0</t>
   </si>
   <si>
+    <t xml:space="preserve">Plantilla Móvil/Web</t>
+  </si>
+  <si>
     <t>MOB1</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Móvil/Web de Login</t>
+  </si>
+  <si>
     <t>MOB2</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Móvil/Web para ver Resumen de Estado</t>
+  </si>
+  <si>
     <t>MOB3</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Móvil/Web para Administrar "Mi expediente"</t>
+  </si>
+  <si>
     <t>MOB4</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Móvil/Web para Realizar Prematrícula</t>
+  </si>
+  <si>
     <t>MOB5</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Móvil/Web para Realizar Matrícula</t>
+  </si>
+  <si>
     <t>MOB6</t>
   </si>
   <si>
+    <t xml:space="preserve">Pantalla Móvil/Web para Consultar "Mis cursos"</t>
+  </si>
+  <si>
     <t>Gateway</t>
   </si>
   <si>
     <t>GTW1</t>
   </si>
   <si>
+    <t xml:space="preserve">Gateway como Punto Único de Entrada</t>
+  </si>
+  <si>
     <t>GTW2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autenticación y Autorización en Gateway</t>
   </si>
 </sst>
 </file>
@@ -514,8 +613,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor theme="7" tint="0.59999389629810485"/>
+        <fgColor indexed="5"/>
+        <bgColor indexed="5"/>
       </patternFill>
     </fill>
     <fill>
@@ -873,6 +972,9 @@
     <xf fontId="0" fillId="10" borderId="4" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf fontId="0" fillId="9" borderId="4" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf fontId="0" fillId="9" borderId="5" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -921,6 +1023,9 @@
     <xf fontId="4" fillId="11" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf fontId="0" fillId="9" borderId="2" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf fontId="6" fillId="0" borderId="12" numFmtId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -966,9 +1071,6 @@
     <xf fontId="6" fillId="0" borderId="10" numFmtId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="9" borderId="4" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf fontId="4" fillId="9" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -979,14 +1081,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="6" fillId="0" borderId="4" numFmtId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="4" fillId="9" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="9" borderId="5" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf fontId="4" fillId="9" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="6" fillId="0" borderId="5" numFmtId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1004,9 +1106,6 @@
     </xf>
     <xf fontId="0" fillId="9" borderId="19" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="9" borderId="11" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1051,7 +1150,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="AskingMansOz" id="{B0EB0FF8-EFF9-D70C-66D6-B6B80F94BA20}" userId="AskingMansOz" providerId="Teamlab"/>
+  <person displayName="AskingMansOz" id="{0AC76D2A-7EE8-23CE-800C-894AC228CA69}" userId="AskingMansOz" providerId="Teamlab"/>
 </personList>
 </file>
 
@@ -1535,7 +1634,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="C4" dT="2026-09-19T09:13:08.03Z" personId="{B0EB0FF8-EFF9-D70C-66D6-B6B80F94BA20}" id="{04CB6911-E216-5FFA-A00E-331AF1FB8FD4}" done="1">
+  <threadedComment ref="C4" dT="2026-09-19T09:13:08.03Z" personId="{0AC76D2A-7EE8-23CE-800C-894AC228CA69}" id="{04CB6911-E216-5FFA-A00E-331AF1FB8FD4}" done="1">
     <text xml:space="preserve">Mide la carga de trabajo del equipo con base en el promedio de puntos acumulados por los integrantes:
 * Verde: Por debajo del promedio (menor carga).
 * Amarillo: En el promedio exacto (carga equilibrada).
@@ -1543,7 +1642,7 @@
 Lo ideal es que la carga de trabajo se mantengan cerca del promedio.
 </text>
   </threadedComment>
-  <threadedComment ref="D4" dT="2026-09-25T19:25:05.93Z" personId="{B0EB0FF8-EFF9-D70C-66D6-B6B80F94BA20}" id="{6A98EA58-EBE2-D560-1FEC-96EE11A8B0CE}" done="1">
+  <threadedComment ref="D4" dT="2026-09-25T19:25:05.93Z" personId="{0AC76D2A-7EE8-23CE-800C-894AC228CA69}" id="{6A98EA58-EBE2-D560-1FEC-96EE11A8B0CE}" done="1">
     <text xml:space="preserve">21.6 x Persona
 </text>
   </threadedComment>
@@ -1556,7 +1655,7 @@
   <cols>
     <col customWidth="1" min="2" max="2" width="33.28125"/>
     <col customWidth="1" min="3" max="3" width="17.140625"/>
-    <col customWidth="1" min="4" max="4" width="49.28125"/>
+    <col customWidth="1" min="4" max="4" width="54.7109375"/>
     <col customWidth="1" min="5" max="5" style="1" width="12.140625"/>
     <col customWidth="1" min="6" max="6" width="27.00390625"/>
     <col customWidth="1" min="7" max="7" width="18.421875"/>
@@ -1590,11 +1689,11 @@
         <v>4</v>
       </c>
       <c r="C4" s="4">
-        <f>SUMIF($F$13:$F$135,B4,$E$13:$E$135)</f>
+        <f t="shared" ref="C4:C8" si="0">SUMIF($F$13:$F$135,B4,$E$13:$E$135)</f>
         <v>21</v>
       </c>
       <c r="D4" s="5">
-        <f>COUNTIF($E$13:$F$135,B4)</f>
+        <f t="shared" ref="D4:D8" si="1">COUNTIF($E$13:$F$135,B4)</f>
         <v>5</v>
       </c>
       <c r="F4" s="6" t="s">
@@ -1606,11 +1705,11 @@
         <v>6</v>
       </c>
       <c r="C5" s="4">
-        <f>SUMIF($F$13:$F$135,B5,$E$13:$E$135)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="D5" s="5">
-        <f>COUNTIF($E$13:$F$135,B5)</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="F5" s="8" t="s">
@@ -1622,11 +1721,11 @@
         <v>8</v>
       </c>
       <c r="C6" s="4">
-        <f>SUMIF($F$13:$F$135,B6,$E$13:$E$135)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="D6" s="5">
-        <f>COUNTIF($E$13:$F$135,B6)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="F6" s="9" t="s">
@@ -1638,11 +1737,11 @@
         <v>10</v>
       </c>
       <c r="C7" s="4">
-        <f>SUMIF($F$13:$F$135,B7,$E$13:$E$135)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="D7" s="5">
-        <f>COUNTIF($E$13:$F$135,B7)</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
     </row>
@@ -1651,11 +1750,11 @@
         <v>11</v>
       </c>
       <c r="C8" s="4">
-        <f>SUMIF($F$13:$F$135,B8,$E$13:$E$135)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="D8" s="11">
-        <f>COUNTIF($E$13:$F$135,B8)</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="H8" s="12"/>
@@ -1738,7 +1837,7 @@
       <c r="C15" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="D15" s="22" t="s">
+      <c r="D15" s="27" t="s">
         <v>25</v>
       </c>
       <c r="E15" s="24">
@@ -1772,59 +1871,59 @@
       </c>
     </row>
     <row r="17" ht="71.25">
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="27" t="s">
+      <c r="D17" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="E17" s="29">
+      <c r="E17" s="30">
         <v>8</v>
       </c>
-      <c r="F17" s="30" t="s">
+      <c r="F17" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="G17" s="31" t="s">
+      <c r="G17" s="32" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="18" ht="42.75">
-      <c r="B18" s="32" t="s">
+      <c r="B18" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="33" t="s">
+      <c r="C18" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="32" t="s">
+      <c r="D18" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="E18" s="34">
-        <v>5</v>
-      </c>
-      <c r="F18" s="35" t="s">
+      <c r="E18" s="35">
+        <v>5</v>
+      </c>
+      <c r="F18" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="G18" s="36" t="s">
+      <c r="G18" s="37" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="19" ht="57">
-      <c r="B19" s="37" t="s">
+      <c r="B19" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="38" t="s">
+      <c r="C19" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="37" t="s">
+      <c r="D19" s="38" t="s">
         <v>34</v>
       </c>
       <c r="E19" s="24">
         <v>5</v>
       </c>
-      <c r="F19" s="39" t="s">
+      <c r="F19" s="40" t="s">
         <v>10</v>
       </c>
       <c r="G19" s="26" t="s">
@@ -1832,19 +1931,19 @@
       </c>
     </row>
     <row r="20" ht="42.75">
-      <c r="B20" s="37" t="s">
+      <c r="B20" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="C20" s="38" t="s">
+      <c r="C20" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="37" t="s">
+      <c r="D20" s="38" t="s">
         <v>36</v>
       </c>
       <c r="E20" s="24">
         <v>5</v>
       </c>
-      <c r="F20" s="39" t="s">
+      <c r="F20" s="40" t="s">
         <v>10</v>
       </c>
       <c r="G20" s="26" t="s">
@@ -1852,19 +1951,19 @@
       </c>
     </row>
     <row r="21" ht="57">
-      <c r="B21" s="37" t="s">
+      <c r="B21" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="38" t="s">
+      <c r="C21" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="D21" s="37" t="s">
+      <c r="D21" s="38" t="s">
         <v>38</v>
       </c>
       <c r="E21" s="24">
         <v>5</v>
       </c>
-      <c r="F21" s="39" t="s">
+      <c r="F21" s="40" t="s">
         <v>8</v>
       </c>
       <c r="G21" s="26" t="s">
@@ -1872,19 +1971,19 @@
       </c>
     </row>
     <row r="22" ht="42.75">
-      <c r="B22" s="37" t="s">
+      <c r="B22" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="38" t="s">
+      <c r="C22" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="D22" s="37" t="s">
+      <c r="D22" s="38" t="s">
         <v>40</v>
       </c>
       <c r="E22" s="24">
         <v>5</v>
       </c>
-      <c r="F22" s="39" t="s">
+      <c r="F22" s="40" t="s">
         <v>8</v>
       </c>
       <c r="G22" s="26" t="s">
@@ -1892,22 +1991,22 @@
       </c>
     </row>
     <row r="23" ht="57">
-      <c r="B23" s="40" t="s">
+      <c r="B23" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="41" t="s">
+      <c r="C23" s="42" t="s">
         <v>41</v>
       </c>
-      <c r="D23" s="40" t="s">
+      <c r="D23" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="E23" s="29">
-        <v>5</v>
-      </c>
-      <c r="F23" s="42" t="s">
+      <c r="E23" s="30">
+        <v>5</v>
+      </c>
+      <c r="F23" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="G23" s="31" t="s">
+      <c r="G23" s="32" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1918,7 +2017,7 @@
       <c r="C24" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="D24" s="17" t="s">
+      <c r="D24" s="44" t="s">
         <v>45</v>
       </c>
       <c r="E24" s="19">
@@ -1927,7 +2026,7 @@
       <c r="F24" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="G24" s="36" t="s">
+      <c r="G24" s="37" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1941,7 +2040,7 @@
       <c r="D25" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="E25" s="43">
+      <c r="E25" s="45">
         <v>5</v>
       </c>
       <c r="F25" s="25" t="s">
@@ -1958,7 +2057,7 @@
       <c r="C26" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="D26" s="44" t="s">
+      <c r="D26" s="46" t="s">
         <v>49</v>
       </c>
       <c r="E26" s="24">
@@ -1981,7 +2080,7 @@
       <c r="D27" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="E27" s="45">
+      <c r="E27" s="47">
         <v>3</v>
       </c>
       <c r="F27" s="25" t="s">
@@ -1992,62 +2091,62 @@
       </c>
     </row>
     <row r="28" ht="57">
-      <c r="B28" s="27" t="s">
+      <c r="B28" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="C28" s="28" t="s">
+      <c r="C28" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="D28" s="27" t="s">
+      <c r="D28" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="E28" s="46">
+      <c r="E28" s="48">
         <v>8</v>
       </c>
-      <c r="F28" s="30" t="s">
+      <c r="F28" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="G28" s="31" t="s">
+      <c r="G28" s="32" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="29" ht="42.75">
-      <c r="B29" s="32" t="s">
+      <c r="B29" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="C29" s="33" t="s">
+      <c r="C29" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="D29" s="32" t="s">
+      <c r="D29" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="E29" s="47">
+      <c r="E29" s="49">
         <v>3</v>
       </c>
-      <c r="F29" s="35" t="s">
+      <c r="F29" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="G29" s="36" t="s">
+      <c r="G29" s="37" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="30" ht="42.75">
-      <c r="B30" s="40" t="s">
+      <c r="B30" s="41" t="s">
         <v>54</v>
       </c>
-      <c r="C30" s="41" t="s">
+      <c r="C30" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="D30" s="40" t="s">
+      <c r="D30" s="41" t="s">
         <v>58</v>
       </c>
-      <c r="E30" s="48">
+      <c r="E30" s="50">
         <v>3</v>
       </c>
-      <c r="F30" s="42" t="s">
+      <c r="F30" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="G30" s="31" t="s">
+      <c r="G30" s="32" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2067,7 +2166,7 @@
       <c r="F31" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="G31" s="36" t="s">
+      <c r="G31" s="37" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2081,7 +2180,7 @@
       <c r="D32" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="E32" s="43">
+      <c r="E32" s="45">
         <v>5</v>
       </c>
       <c r="F32" s="25" t="s">
@@ -2092,42 +2191,42 @@
       </c>
     </row>
     <row r="33" ht="42.75">
-      <c r="B33" s="27" t="s">
+      <c r="B33" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="C33" s="28" t="s">
+      <c r="C33" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="27" t="s">
+      <c r="D33" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="48">
+      <c r="E33" s="50">
         <v>3</v>
       </c>
-      <c r="F33" s="30" t="s">
+      <c r="F33" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="G33" s="31" t="s">
+      <c r="G33" s="32" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="34" ht="57">
-      <c r="B34" s="49" t="s">
+      <c r="B34" s="51" t="s">
         <v>66</v>
       </c>
-      <c r="C34" s="50" t="s">
+      <c r="C34" s="52" t="s">
         <v>67</v>
       </c>
-      <c r="D34" s="49" t="s">
+      <c r="D34" s="51" t="s">
         <v>68</v>
       </c>
-      <c r="E34" s="51">
+      <c r="E34" s="53">
         <v>2</v>
       </c>
-      <c r="F34" s="52" t="s">
+      <c r="F34" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="G34" s="53" t="s">
+      <c r="G34" s="55" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2152,429 +2251,561 @@
       </c>
     </row>
     <row r="36" ht="57">
-      <c r="B36" s="54" t="s">
+      <c r="B36" s="56" t="s">
         <v>70</v>
       </c>
-      <c r="C36" s="55" t="s">
+      <c r="C36" s="57" t="s">
         <v>71</v>
       </c>
-      <c r="D36" s="56"/>
-      <c r="E36" s="57"/>
+      <c r="D36" s="58" t="s">
+        <v>72</v>
+      </c>
+      <c r="E36" s="59">
+        <v>3</v>
+      </c>
       <c r="F36" s="20"/>
       <c r="G36" s="21"/>
     </row>
     <row r="37" ht="57">
-      <c r="B37" s="58" t="s">
+      <c r="B37" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C37" s="59" t="s">
-        <v>72</v>
-      </c>
-      <c r="D37" s="22"/>
-      <c r="E37" s="60"/>
+      <c r="C37" s="60" t="s">
+        <v>73</v>
+      </c>
+      <c r="D37" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="E37" s="61">
+        <v>3</v>
+      </c>
       <c r="F37" s="25"/>
       <c r="G37" s="26"/>
     </row>
     <row r="38" ht="57">
-      <c r="B38" s="58" t="s">
+      <c r="B38" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C38" s="59" t="s">
-        <v>73</v>
-      </c>
-      <c r="D38" s="22"/>
-      <c r="E38" s="61"/>
+      <c r="C38" s="60" t="s">
+        <v>75</v>
+      </c>
+      <c r="D38" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="E38" s="62">
+        <v>3</v>
+      </c>
       <c r="F38" s="25"/>
       <c r="G38" s="26"/>
     </row>
     <row r="39" ht="57">
-      <c r="B39" s="58" t="s">
+      <c r="B39" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C39" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="D39" s="22"/>
-      <c r="E39" s="62"/>
+      <c r="C39" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D39" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="E39" s="63">
+        <v>5</v>
+      </c>
       <c r="F39" s="25"/>
       <c r="G39" s="26"/>
     </row>
     <row r="40" ht="57">
-      <c r="B40" s="58" t="s">
+      <c r="B40" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C40" s="59" t="s">
-        <v>75</v>
-      </c>
-      <c r="D40" s="22"/>
-      <c r="E40" s="60"/>
+      <c r="C40" s="60" t="s">
+        <v>79</v>
+      </c>
+      <c r="D40" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="E40" s="61">
+        <v>5</v>
+      </c>
       <c r="F40" s="25"/>
       <c r="G40" s="26"/>
     </row>
     <row r="41" ht="57">
-      <c r="B41" s="58" t="s">
+      <c r="B41" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C41" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="D41" s="22"/>
-      <c r="E41" s="61"/>
+      <c r="C41" s="60" t="s">
+        <v>81</v>
+      </c>
+      <c r="D41" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="E41" s="62">
+        <v>5</v>
+      </c>
       <c r="F41" s="25"/>
       <c r="G41" s="26"/>
     </row>
     <row r="42" ht="57">
-      <c r="B42" s="58" t="s">
+      <c r="B42" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C42" s="59" t="s">
-        <v>77</v>
-      </c>
-      <c r="D42" s="22"/>
-      <c r="E42" s="60"/>
+      <c r="C42" s="60" t="s">
+        <v>83</v>
+      </c>
+      <c r="D42" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="E42" s="61">
+        <v>5</v>
+      </c>
       <c r="F42" s="25"/>
       <c r="G42" s="26"/>
     </row>
     <row r="43" ht="57">
-      <c r="B43" s="58" t="s">
+      <c r="B43" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C43" s="59" t="s">
-        <v>78</v>
-      </c>
-      <c r="D43" s="22"/>
-      <c r="E43" s="61"/>
+      <c r="C43" s="60" t="s">
+        <v>85</v>
+      </c>
+      <c r="D43" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="E43" s="62">
+        <v>5</v>
+      </c>
       <c r="F43" s="25"/>
       <c r="G43" s="26"/>
     </row>
     <row r="44" ht="57">
-      <c r="B44" s="58" t="s">
+      <c r="B44" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C44" s="59" t="s">
-        <v>79</v>
-      </c>
-      <c r="D44" s="22"/>
-      <c r="E44" s="60"/>
+      <c r="C44" s="60" t="s">
+        <v>87</v>
+      </c>
+      <c r="D44" s="27" t="s">
+        <v>88</v>
+      </c>
+      <c r="E44" s="61">
+        <v>5</v>
+      </c>
       <c r="F44" s="25"/>
       <c r="G44" s="26"/>
     </row>
     <row r="45" ht="57">
-      <c r="B45" s="58" t="s">
+      <c r="B45" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C45" s="59" t="s">
-        <v>80</v>
-      </c>
-      <c r="D45" s="22"/>
-      <c r="E45" s="61"/>
+      <c r="C45" s="60" t="s">
+        <v>89</v>
+      </c>
+      <c r="D45" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="E45" s="62">
+        <v>5</v>
+      </c>
       <c r="F45" s="25"/>
       <c r="G45" s="26"/>
     </row>
     <row r="46" ht="57">
-      <c r="B46" s="58" t="s">
+      <c r="B46" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C46" s="59" t="s">
-        <v>81</v>
-      </c>
-      <c r="D46" s="22"/>
-      <c r="E46" s="62"/>
+      <c r="C46" s="60" t="s">
+        <v>91</v>
+      </c>
+      <c r="D46" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="E46" s="63">
+        <v>5</v>
+      </c>
       <c r="F46" s="25"/>
       <c r="G46" s="26"/>
     </row>
     <row r="47" ht="57">
-      <c r="B47" s="58" t="s">
+      <c r="B47" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C47" s="59" t="s">
-        <v>82</v>
-      </c>
-      <c r="D47" s="22"/>
-      <c r="E47" s="60"/>
+      <c r="C47" s="60" t="s">
+        <v>93</v>
+      </c>
+      <c r="D47" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="E47" s="61">
+        <v>5</v>
+      </c>
       <c r="F47" s="25"/>
       <c r="G47" s="26"/>
     </row>
     <row r="48" ht="57">
-      <c r="B48" s="58" t="s">
+      <c r="B48" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C48" s="59" t="s">
-        <v>83</v>
-      </c>
-      <c r="D48" s="22"/>
-      <c r="E48" s="61"/>
+      <c r="C48" s="60" t="s">
+        <v>95</v>
+      </c>
+      <c r="D48" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="E48" s="62">
+        <v>5</v>
+      </c>
       <c r="F48" s="25"/>
       <c r="G48" s="26"/>
     </row>
     <row r="49" ht="57">
-      <c r="B49" s="58" t="s">
+      <c r="B49" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C49" s="59" t="s">
-        <v>84</v>
-      </c>
-      <c r="D49" s="22"/>
-      <c r="E49" s="60"/>
+      <c r="C49" s="60" t="s">
+        <v>97</v>
+      </c>
+      <c r="D49" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="E49" s="61">
+        <v>5</v>
+      </c>
       <c r="F49" s="25"/>
       <c r="G49" s="26"/>
     </row>
     <row r="50" ht="57">
-      <c r="B50" s="58" t="s">
+      <c r="B50" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C50" s="59" t="s">
-        <v>85</v>
-      </c>
-      <c r="D50" s="22"/>
-      <c r="E50" s="60"/>
+      <c r="C50" s="60" t="s">
+        <v>99</v>
+      </c>
+      <c r="D50" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="E50" s="61">
+        <v>5</v>
+      </c>
       <c r="F50" s="25"/>
       <c r="G50" s="26"/>
     </row>
     <row r="51" ht="57">
-      <c r="B51" s="58" t="s">
+      <c r="B51" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C51" s="59" t="s">
-        <v>86</v>
-      </c>
-      <c r="D51" s="22"/>
-      <c r="E51" s="61"/>
+      <c r="C51" s="60" t="s">
+        <v>101</v>
+      </c>
+      <c r="D51" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="E51" s="62">
+        <v>5</v>
+      </c>
       <c r="F51" s="25"/>
       <c r="G51" s="26"/>
     </row>
     <row r="52" ht="57">
-      <c r="B52" s="58" t="s">
+      <c r="B52" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C52" s="59" t="s">
-        <v>87</v>
-      </c>
-      <c r="D52" s="22"/>
-      <c r="E52" s="62"/>
+      <c r="C52" s="60" t="s">
+        <v>103</v>
+      </c>
+      <c r="D52" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="E52" s="63">
+        <v>5</v>
+      </c>
       <c r="F52" s="25"/>
       <c r="G52" s="26"/>
     </row>
     <row r="53" ht="57">
-      <c r="B53" s="58" t="s">
+      <c r="B53" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C53" s="59" t="s">
-        <v>88</v>
-      </c>
-      <c r="D53" s="22"/>
-      <c r="E53" s="60"/>
+      <c r="C53" s="60" t="s">
+        <v>105</v>
+      </c>
+      <c r="D53" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="E53" s="61">
+        <v>3</v>
+      </c>
       <c r="F53" s="25"/>
       <c r="G53" s="26"/>
     </row>
     <row r="54" ht="57">
-      <c r="B54" s="58" t="s">
+      <c r="B54" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C54" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="D54" s="22"/>
-      <c r="E54" s="61"/>
+      <c r="C54" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="D54" s="27" t="s">
+        <v>108</v>
+      </c>
+      <c r="E54" s="62">
+        <v>3</v>
+      </c>
       <c r="F54" s="25"/>
       <c r="G54" s="26"/>
     </row>
     <row r="55" ht="57">
-      <c r="B55" s="58" t="s">
+      <c r="B55" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C55" s="59" t="s">
-        <v>90</v>
-      </c>
-      <c r="D55" s="22"/>
-      <c r="E55" s="60"/>
+      <c r="C55" s="60" t="s">
+        <v>109</v>
+      </c>
+      <c r="D55" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="E55" s="61">
+        <v>5</v>
+      </c>
       <c r="F55" s="25"/>
       <c r="G55" s="26"/>
     </row>
     <row r="56" ht="57">
-      <c r="B56" s="58" t="s">
+      <c r="B56" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C56" s="59" t="s">
-        <v>91</v>
-      </c>
-      <c r="D56" s="22"/>
-      <c r="E56" s="62"/>
+      <c r="C56" s="60" t="s">
+        <v>111</v>
+      </c>
+      <c r="D56" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="E56" s="63">
+        <v>5</v>
+      </c>
       <c r="F56" s="25"/>
       <c r="G56" s="26"/>
     </row>
     <row r="57" ht="57">
-      <c r="B57" s="58" t="s">
+      <c r="B57" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C57" s="59" t="s">
-        <v>92</v>
-      </c>
-      <c r="D57" s="22"/>
-      <c r="E57" s="60"/>
+      <c r="C57" s="60" t="s">
+        <v>113</v>
+      </c>
+      <c r="D57" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="E57" s="61">
+        <v>3</v>
+      </c>
       <c r="F57" s="25"/>
       <c r="G57" s="26"/>
     </row>
     <row r="58" ht="57">
-      <c r="B58" s="58" t="s">
+      <c r="B58" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="C58" s="59" t="s">
-        <v>93</v>
-      </c>
-      <c r="D58" s="22"/>
-      <c r="E58" s="61"/>
+      <c r="C58" s="60" t="s">
+        <v>115</v>
+      </c>
+      <c r="D58" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="E58" s="62">
+        <v>2</v>
+      </c>
       <c r="F58" s="25"/>
       <c r="G58" s="26"/>
     </row>
     <row r="59" ht="57">
-      <c r="B59" s="63" t="s">
+      <c r="B59" s="28" t="s">
         <v>70</v>
       </c>
       <c r="C59" s="64" t="s">
-        <v>94</v>
-      </c>
-      <c r="D59" s="27"/>
-      <c r="E59" s="65"/>
-      <c r="F59" s="30"/>
-      <c r="G59" s="31"/>
-    </row>
-    <row r="60" s="66" customFormat="1" ht="57">
-      <c r="B60" s="67" t="s">
+        <v>117</v>
+      </c>
+      <c r="D59" s="65" t="s">
+        <v>118</v>
+      </c>
+      <c r="E59" s="66">
+        <v>3</v>
+      </c>
+      <c r="F59" s="31"/>
+      <c r="G59" s="32"/>
+    </row>
+    <row r="60" s="67" customFormat="1" ht="57">
+      <c r="B60" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="C60" s="67" t="s">
+      <c r="C60" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="D60" s="67" t="s">
-        <v>95</v>
-      </c>
-      <c r="E60" s="68" t="s">
+      <c r="D60" s="68" t="s">
+        <v>119</v>
+      </c>
+      <c r="E60" s="69" t="s">
         <v>16</v>
       </c>
-      <c r="F60" s="67" t="s">
+      <c r="F60" s="68" t="s">
         <v>17</v>
       </c>
-      <c r="G60" s="68" t="s">
+      <c r="G60" s="69" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="61" s="66" customFormat="1" ht="57">
-      <c r="A61" s="69"/>
-      <c r="B61" s="54" t="s">
-        <v>96</v>
-      </c>
-      <c r="C61" s="55" t="s">
-        <v>97</v>
-      </c>
-      <c r="D61" s="70"/>
-      <c r="E61" s="57"/>
-      <c r="F61" s="55"/>
+    <row r="61" s="67" customFormat="1" ht="57">
+      <c r="A61" s="70"/>
+      <c r="B61" s="56" t="s">
+        <v>120</v>
+      </c>
+      <c r="C61" s="57" t="s">
+        <v>121</v>
+      </c>
+      <c r="D61" s="71" t="s">
+        <v>122</v>
+      </c>
+      <c r="E61" s="59">
+        <v>3</v>
+      </c>
+      <c r="F61" s="57"/>
       <c r="G61" s="21"/>
     </row>
-    <row r="62" s="66" customFormat="1" ht="57">
-      <c r="A62" s="71"/>
-      <c r="B62" s="58" t="s">
-        <v>96</v>
-      </c>
-      <c r="C62" s="59" t="s">
-        <v>98</v>
-      </c>
-      <c r="D62" s="72"/>
-      <c r="E62" s="60"/>
-      <c r="F62" s="59"/>
+    <row r="62" s="67" customFormat="1" ht="57">
+      <c r="A62" s="70"/>
+      <c r="B62" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="C62" s="60" t="s">
+        <v>123</v>
+      </c>
+      <c r="D62" s="72" t="s">
+        <v>124</v>
+      </c>
+      <c r="E62" s="61">
+        <v>3</v>
+      </c>
+      <c r="F62" s="60"/>
       <c r="G62" s="26"/>
     </row>
-    <row r="63" s="66" customFormat="1" ht="57">
-      <c r="A63" s="71"/>
-      <c r="B63" s="58" t="s">
-        <v>96</v>
-      </c>
-      <c r="C63" s="59" t="s">
-        <v>99</v>
-      </c>
-      <c r="D63" s="72"/>
-      <c r="E63" s="60"/>
-      <c r="F63" s="59"/>
+    <row r="63" s="67" customFormat="1" ht="57">
+      <c r="A63" s="70"/>
+      <c r="B63" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="C63" s="60" t="s">
+        <v>125</v>
+      </c>
+      <c r="D63" s="72" t="s">
+        <v>126</v>
+      </c>
+      <c r="E63" s="61">
+        <v>3</v>
+      </c>
+      <c r="F63" s="60"/>
       <c r="G63" s="26"/>
     </row>
-    <row r="64" s="66" customFormat="1" ht="57">
-      <c r="A64" s="71"/>
-      <c r="B64" s="58" t="s">
-        <v>96</v>
-      </c>
-      <c r="C64" s="59" t="s">
-        <v>100</v>
-      </c>
-      <c r="D64" s="72"/>
-      <c r="E64" s="60"/>
-      <c r="F64" s="59"/>
+    <row r="64" s="67" customFormat="1" ht="57">
+      <c r="A64" s="70"/>
+      <c r="B64" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="C64" s="60" t="s">
+        <v>127</v>
+      </c>
+      <c r="D64" s="72" t="s">
+        <v>128</v>
+      </c>
+      <c r="E64" s="61">
+        <v>3</v>
+      </c>
+      <c r="F64" s="60"/>
       <c r="G64" s="26"/>
     </row>
-    <row r="65" s="66" customFormat="1" ht="57">
-      <c r="A65" s="71"/>
-      <c r="B65" s="58" t="s">
-        <v>96</v>
-      </c>
-      <c r="C65" s="59" t="s">
-        <v>101</v>
-      </c>
-      <c r="D65" s="72"/>
-      <c r="E65" s="60"/>
-      <c r="F65" s="59"/>
+    <row r="65" s="67" customFormat="1" ht="57">
+      <c r="A65" s="70"/>
+      <c r="B65" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="C65" s="60" t="s">
+        <v>129</v>
+      </c>
+      <c r="D65" s="72" t="s">
+        <v>130</v>
+      </c>
+      <c r="E65" s="61">
+        <v>3</v>
+      </c>
+      <c r="F65" s="60"/>
       <c r="G65" s="26"/>
     </row>
-    <row r="66" s="66" customFormat="1" ht="57">
-      <c r="A66" s="71"/>
-      <c r="B66" s="58" t="s">
-        <v>96</v>
-      </c>
-      <c r="C66" s="59" t="s">
-        <v>102</v>
-      </c>
-      <c r="D66" s="72"/>
-      <c r="E66" s="60"/>
-      <c r="F66" s="59"/>
+    <row r="66" s="67" customFormat="1" ht="57">
+      <c r="A66" s="70"/>
+      <c r="B66" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="C66" s="60" t="s">
+        <v>131</v>
+      </c>
+      <c r="D66" s="72" t="s">
+        <v>132</v>
+      </c>
+      <c r="E66" s="61">
+        <v>3</v>
+      </c>
+      <c r="F66" s="60"/>
       <c r="G66" s="26"/>
     </row>
-    <row r="67" s="66" customFormat="1" ht="57">
-      <c r="A67" s="71"/>
-      <c r="B67" s="63" t="s">
-        <v>96</v>
+    <row r="67" s="67" customFormat="1" ht="57">
+      <c r="A67" s="70"/>
+      <c r="B67" s="28" t="s">
+        <v>120</v>
       </c>
       <c r="C67" s="64" t="s">
-        <v>103</v>
-      </c>
-      <c r="D67" s="73"/>
-      <c r="E67" s="65"/>
+        <v>133</v>
+      </c>
+      <c r="D67" s="73" t="s">
+        <v>134</v>
+      </c>
+      <c r="E67" s="66">
+        <v>3</v>
+      </c>
       <c r="F67" s="64"/>
-      <c r="G67" s="31"/>
-    </row>
-    <row r="68" s="66" customFormat="1" ht="57">
-      <c r="A68" s="71"/>
+      <c r="G67" s="32"/>
+    </row>
+    <row r="68" s="67" customFormat="1" ht="57">
+      <c r="A68" s="70"/>
       <c r="B68" s="74" t="s">
-        <v>104</v>
-      </c>
-      <c r="C68" s="33" t="s">
-        <v>105</v>
-      </c>
-      <c r="D68" s="75"/>
-      <c r="E68" s="57"/>
-      <c r="F68" s="33"/>
+        <v>135</v>
+      </c>
+      <c r="C68" s="34" t="s">
+        <v>136</v>
+      </c>
+      <c r="D68" s="75" t="s">
+        <v>137</v>
+      </c>
+      <c r="E68" s="59">
+        <v>5</v>
+      </c>
+      <c r="F68" s="34"/>
       <c r="G68" s="21"/>
     </row>
-    <row r="69" s="66" customFormat="1" ht="57">
-      <c r="A69" s="71"/>
-      <c r="B69" s="76" t="s">
-        <v>104</v>
-      </c>
-      <c r="C69" s="41" t="s">
-        <v>106</v>
-      </c>
-      <c r="D69" s="40"/>
-      <c r="E69" s="65"/>
-      <c r="F69" s="41"/>
-      <c r="G69" s="31"/>
+    <row r="69" s="67" customFormat="1" ht="57">
+      <c r="A69" s="70"/>
+      <c r="B69" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="C69" s="42" t="s">
+        <v>138</v>
+      </c>
+      <c r="D69" s="76" t="s">
+        <v>139</v>
+      </c>
+      <c r="E69" s="66">
+        <v>5</v>
+      </c>
+      <c r="F69" s="42"/>
+      <c r="G69" s="32"/>
     </row>
     <row r="70" ht="14.25">
       <c r="D70" s="77" t="s">
@@ -2582,7 +2813,7 @@
       </c>
       <c r="E70" s="78">
         <f>SUM(E13:E34,E36:E59,E61:E69)</f>
-        <v>108</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -2593,47 +2824,47 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G36:G39">
-    <cfRule type="containsText" priority="2" text="En Desarrollo">
+    <cfRule type="containsText" priority="13" text="En Desarrollo">
       <formula>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G40:G42">
-    <cfRule type="containsText" priority="2" text="En Desarrollo">
+    <cfRule type="containsText" priority="14" text="En Desarrollo">
       <formula>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G43:G45">
-    <cfRule type="containsText" priority="2" text="En Desarrollo">
+    <cfRule type="containsText" priority="15" text="En Desarrollo">
       <formula>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G46:G48">
-    <cfRule type="containsText" priority="2" text="En Desarrollo">
+    <cfRule type="containsText" priority="16" text="En Desarrollo">
       <formula>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G49:G51">
-    <cfRule type="containsText" priority="2" text="En Desarrollo">
+    <cfRule type="containsText" priority="17" text="En Desarrollo">
       <formula>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G52:G54">
-    <cfRule type="containsText" priority="2" text="En Desarrollo">
+    <cfRule type="containsText" priority="18" text="En Desarrollo">
       <formula>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G55:G57">
-    <cfRule type="containsText" priority="2" text="En Desarrollo">
+    <cfRule type="containsText" priority="19" text="En Desarrollo">
       <formula>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G58:G59">
-    <cfRule type="containsText" priority="2" text="En Desarrollo">
+    <cfRule type="containsText" priority="20" text="En Desarrollo">
       <formula>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G61:G69">
-    <cfRule type="containsText" priority="2" text="En Desarrollo">
+    <cfRule type="containsText" priority="21" text="En Desarrollo">
       <formula>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2649,7 +2880,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{E274936B-A901-4A89-A651-14C6EE3DC4CF}">
+          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{7E21A8D1-4233-42EE-A5DF-FAD1CE5DEE89}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -2660,7 +2891,7 @@
           <xm:sqref>E13:E34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{A46ABE3F-E97C-4686-A784-82CABC18EABB}">
+          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{FE517BA7-2A8B-49BA-A909-4E76569A73DA}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -2677,7 +2908,7 @@
           <xm:sqref>E13:E34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{C22A426A-E4E1-4067-A456-B69114B10A37}">
+          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{7BAC9785-03FC-4822-AEFF-69458A015822}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -2695,7 +2926,7 @@
           <xm:sqref>E13:E34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{FD37D9E4-8049-4AA6-A35A-1C99D7F5D051}">
+          <x14:cfRule type="cellIs" priority="9" operator="between" id="{91B6724D-75EE-42CA-B330-3ABA75EC12C5}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -2713,7 +2944,7 @@
           <xm:sqref>E13:E34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{86D641FD-EA4D-4BCF-ADBD-C1EFD6C2705F}">
+          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{8A951659-27A9-43E3-9D0E-F25529B17597}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -2730,7 +2961,7 @@
           <xm:sqref>E13:E34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="aboveAverage" priority="7" stdDev="0" id="{978B431C-8EE9-4E03-9B95-2B09AF1064B9}">
+          <x14:cfRule type="aboveAverage" priority="7" stdDev="0" id="{25ABD6C5-5FF9-484D-9C49-4AE287E998A7}">
             <x14:dxf>
               <font>
                 <color rgb="FF9C0006"/>
@@ -2746,7 +2977,7 @@
           <xm:sqref>C4:C8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="aboveAverage" priority="6" aboveAverage="0" stdDev="0" id="{23D6DF3B-FEC4-41F1-B73F-351061E947F3}">
+          <x14:cfRule type="aboveAverage" priority="6" aboveAverage="0" stdDev="0" id="{D75F4D26-7F91-4CB6-99C8-1C70795AAA9A}">
             <x14:dxf>
               <font>
                 <color rgb="FF006100"/>
@@ -2762,7 +2993,7 @@
           <xm:sqref>C4:C8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="5" operator="lessThan" id="{C79AE3AB-D85E-494F-8E5D-3673FFA38655}">
+          <x14:cfRule type="cellIs" priority="5" operator="lessThan" id="{DAEDCE5B-6564-4A27-AC2F-70A51C158E67}">
             <xm:f>5</xm:f>
             <x14:dxf>
               <font>
@@ -2779,7 +3010,7 @@
           <xm:sqref>E34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{F5E51FFC-62B4-4C39-9565-95D4517DD94A}">
+          <x14:cfRule type="cellIs" priority="22" operator="equal" id="{A6E8FE57-AED4-45F9-A105-8704D552C3A9}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -2790,7 +3021,7 @@
           <xm:sqref>E36:E39</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{6A6465C9-49E5-4D5B-8BD7-440246B08655}">
+          <x14:cfRule type="cellIs" priority="23" operator="lessThanOrEqual" id="{1ECF257F-C399-4D5D-BF04-9FC639EAEF65}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -2807,7 +3038,7 @@
           <xm:sqref>E36:E39</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{80FB6721-AA9E-442C-9662-2432AF913B59}">
+          <x14:cfRule type="cellIs" priority="24" operator="notBetween" id="{AD80A781-D6EE-4F7A-9E17-E7173C08C7D6}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -2825,7 +3056,7 @@
           <xm:sqref>E36:E39</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{303CFF23-EA61-4061-B27D-D1BA84FE3E63}">
+          <x14:cfRule type="cellIs" priority="25" operator="between" id="{0C0D6CD7-98E3-4312-AFA7-088E8980DDA4}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -2843,7 +3074,7 @@
           <xm:sqref>E36:E39</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{694538A7-6E5E-4642-A8DC-39238937C25B}">
+          <x14:cfRule type="cellIs" priority="26" operator="greaterThanOrEqual" id="{46DF6C61-984B-4BAA-8D63-59AB84B6512F}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -2860,7 +3091,7 @@
           <xm:sqref>E36:E39</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{7EC868EC-8927-4D5D-84F7-C6963655DDAF}">
+          <x14:cfRule type="cellIs" priority="27" operator="equal" id="{E218CEEC-D5EE-49D4-A7E0-9624805941F1}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -2871,7 +3102,7 @@
           <xm:sqref>E40:E41</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{304CD281-4467-4823-AF92-3DC19F73B7FD}">
+          <x14:cfRule type="cellIs" priority="28" operator="lessThanOrEqual" id="{950B2D12-CA72-40FF-83F4-10B5861DD817}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -2888,7 +3119,7 @@
           <xm:sqref>E40:E41</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{F15C9EB0-75BB-47E7-9969-32FAEEBFAF00}">
+          <x14:cfRule type="cellIs" priority="29" operator="notBetween" id="{A9DB20AD-C93E-4DAB-B2BF-DBDD98313DC2}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -2906,7 +3137,7 @@
           <xm:sqref>E40:E41</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{BCFFA081-FE88-4AA4-9D6C-6EAAED39F63A}">
+          <x14:cfRule type="cellIs" priority="30" operator="between" id="{5130AE10-D9FC-4AD8-98B7-AF04EAA8FF9C}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -2924,7 +3155,7 @@
           <xm:sqref>E40:E41</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{84E33312-D897-4F0D-B52C-55F7BFAFB090}">
+          <x14:cfRule type="cellIs" priority="31" operator="greaterThanOrEqual" id="{F185C72F-D42A-4837-B2DB-EE67F7E7E835}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -2941,7 +3172,7 @@
           <xm:sqref>E40:E41</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{81CE7598-2514-4DE3-BAF6-0916A60FC8CB}">
+          <x14:cfRule type="cellIs" priority="32" operator="equal" id="{C8B9BAD3-34F3-4B05-9E53-1F9211BC3D92}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -2952,7 +3183,7 @@
           <xm:sqref>E42:E43</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{5469A41A-3190-448E-8DC8-1FA823C01761}">
+          <x14:cfRule type="cellIs" priority="33" operator="lessThanOrEqual" id="{85B28714-A67E-44FC-AB91-080B69ADB187}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -2969,7 +3200,7 @@
           <xm:sqref>E42:E43</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{04578C98-13B3-4018-B1C0-C2995134C4F6}">
+          <x14:cfRule type="cellIs" priority="34" operator="notBetween" id="{A5657FC9-8568-492F-88E7-436941794B9B}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -2987,7 +3218,7 @@
           <xm:sqref>E42:E43</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{5E80B251-2D24-463F-8574-8B3F94485234}">
+          <x14:cfRule type="cellIs" priority="35" operator="between" id="{48C63E37-2392-47CA-A8AB-A13E89865D5B}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -3005,7 +3236,7 @@
           <xm:sqref>E42:E43</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{36A4FBF5-C517-4E34-9B62-B8EA3C772CC8}">
+          <x14:cfRule type="cellIs" priority="36" operator="greaterThanOrEqual" id="{25798A48-EB9B-4CE2-BF2E-4D17323626BF}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -3022,7 +3253,7 @@
           <xm:sqref>E42:E43</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{EE8BA9D4-F0B9-4E61-B3BB-F6F38B2E9FD3}">
+          <x14:cfRule type="cellIs" priority="37" operator="equal" id="{DC897235-86CC-4549-8720-6BFCAFF2FDAF}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3033,7 +3264,7 @@
           <xm:sqref>E44:E46</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{32CFB9B5-290F-447F-A604-09531E1CA592}">
+          <x14:cfRule type="cellIs" priority="38" operator="lessThanOrEqual" id="{EC4F63FD-BCF8-4A7B-97A2-97E6E08993E3}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3050,7 +3281,7 @@
           <xm:sqref>E44:E46</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{B82F99AE-16A7-4CC4-8D43-B7C40AD63D18}">
+          <x14:cfRule type="cellIs" priority="39" operator="notBetween" id="{F84334BC-DC53-4F23-AAD4-15AB96F5FC5C}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -3068,7 +3299,7 @@
           <xm:sqref>E44:E46</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{2946943C-6013-4B7B-BA22-C72E4E25307C}">
+          <x14:cfRule type="cellIs" priority="40" operator="between" id="{12222348-BEE9-40CC-A591-1555647D40D2}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -3086,7 +3317,7 @@
           <xm:sqref>E44:E46</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{A735B590-05F3-44F5-9D30-91E625DE4DAA}">
+          <x14:cfRule type="cellIs" priority="41" operator="greaterThanOrEqual" id="{9FE79E67-497F-4F89-A1BD-963279640C5F}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -3103,7 +3334,7 @@
           <xm:sqref>E44:E46</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{718E3598-83F6-4C54-AFA7-406F316A3EAE}">
+          <x14:cfRule type="cellIs" priority="42" operator="equal" id="{337D494A-49AD-4492-9EB1-088A8858E6F5}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3114,7 +3345,7 @@
           <xm:sqref>E47:E48</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{DAC7F99C-B5B7-4A02-9D7B-286981C4C33B}">
+          <x14:cfRule type="cellIs" priority="43" operator="lessThanOrEqual" id="{985D9E96-19AD-4EA5-ABCA-D9013B98D68A}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3131,7 +3362,7 @@
           <xm:sqref>E47:E48</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{01D67E10-76CA-4205-91C2-3D20F697F853}">
+          <x14:cfRule type="cellIs" priority="44" operator="notBetween" id="{9F149856-F0EF-47E0-951F-D43B3F4D4DC7}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -3149,7 +3380,7 @@
           <xm:sqref>E47:E48</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{C60E3951-7B09-4EEE-9EC8-4CC4AFC0B4BF}">
+          <x14:cfRule type="cellIs" priority="45" operator="between" id="{D6180286-76F6-4746-87AD-6F55FFB439FD}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -3167,7 +3398,7 @@
           <xm:sqref>E47:E48</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{CB048B9A-AC12-49F4-B865-D0BA9A24E584}">
+          <x14:cfRule type="cellIs" priority="46" operator="greaterThanOrEqual" id="{E7BAFEFB-8356-4D3E-A736-B63AF8B1AF2B}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -3184,7 +3415,7 @@
           <xm:sqref>E47:E48</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{965F935D-213D-40B0-A5DE-E586B9058563}">
+          <x14:cfRule type="cellIs" priority="47" operator="equal" id="{60BC18CE-B70B-4F93-94EA-3B98ADCF1128}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3195,7 +3426,7 @@
           <xm:sqref>E49</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{B8ECB341-B8ED-4762-96CE-D0916D217356}">
+          <x14:cfRule type="cellIs" priority="48" operator="lessThanOrEqual" id="{4BFF66E3-7E30-415B-8913-A9A8838B7BD0}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3212,7 +3443,7 @@
           <xm:sqref>E49</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{B68D501F-ACF9-4EC9-83B2-FE11F4D422A8}">
+          <x14:cfRule type="cellIs" priority="49" operator="notBetween" id="{96342C7A-D299-4203-A969-1ED41182BB58}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -3230,7 +3461,7 @@
           <xm:sqref>E49</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{283BE597-0CD8-4CCE-AD25-2D0D2F62DCAB}">
+          <x14:cfRule type="cellIs" priority="50" operator="between" id="{827A52A5-C4F0-4854-AFBD-F5FDEB6BB91D}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -3248,7 +3479,7 @@
           <xm:sqref>E49</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{3E9FC6C3-E19A-4B71-BE49-D269546D5EF6}">
+          <x14:cfRule type="cellIs" priority="51" operator="greaterThanOrEqual" id="{953B567B-E1EC-4942-AD27-863BDD141286}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -3265,7 +3496,7 @@
           <xm:sqref>E49</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{3C43090E-501F-4071-9818-6BA2DFE4304B}">
+          <x14:cfRule type="cellIs" priority="52" operator="equal" id="{1FA5A7F7-2232-4EE6-A8EE-7D586A9DC555}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3276,7 +3507,7 @@
           <xm:sqref>E50:E52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{D8B7B628-3232-4547-BFD4-E73BA1CACA90}">
+          <x14:cfRule type="cellIs" priority="53" operator="lessThanOrEqual" id="{8B71249B-2898-4BF5-BAE9-53E6B8EE8923}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3293,7 +3524,7 @@
           <xm:sqref>E50:E52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{46E9D17D-20BB-4107-BCC8-3315C5A5D366}">
+          <x14:cfRule type="cellIs" priority="54" operator="notBetween" id="{16E8D38C-C831-4496-931F-0F48F2370331}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -3311,7 +3542,7 @@
           <xm:sqref>E50:E52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{E8BFEE90-7E12-418E-8B34-E593F166AA6F}">
+          <x14:cfRule type="cellIs" priority="55" operator="between" id="{982DBF48-0C5F-422D-B02C-05936D105AEE}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -3329,7 +3560,7 @@
           <xm:sqref>E50:E52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{1081FCF0-3EB0-42DC-84B1-7761ACE4D09C}">
+          <x14:cfRule type="cellIs" priority="56" operator="greaterThanOrEqual" id="{4FDA9EDC-E5BA-40A0-AC43-2C009D4E3C90}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -3346,7 +3577,7 @@
           <xm:sqref>E50:E52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{16F4EE3E-7C14-41CF-888F-EC80BDCE1773}">
+          <x14:cfRule type="cellIs" priority="57" operator="equal" id="{4EB9FBA7-12B3-4197-835F-0A244708E625}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3357,7 +3588,7 @@
           <xm:sqref>E53:E54</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{B9D74BD9-A494-476D-A3A5-08D85DE28473}">
+          <x14:cfRule type="cellIs" priority="58" operator="lessThanOrEqual" id="{E48C2899-F5E1-4C1F-AA46-661521D8F44F}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3374,7 +3605,7 @@
           <xm:sqref>E53:E54</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{8A9F5ECD-07EB-4575-AE8F-1C7A65EF14C4}">
+          <x14:cfRule type="cellIs" priority="59" operator="notBetween" id="{F78DC1E6-7ABA-4CA2-9176-65EC0F9AF59B}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -3392,7 +3623,7 @@
           <xm:sqref>E53:E54</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{DB0FDA59-4EB8-45F3-B13E-AA2ECE2652A2}">
+          <x14:cfRule type="cellIs" priority="60" operator="between" id="{73893DF2-F883-40E1-93A0-7534A4515E89}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -3410,7 +3641,7 @@
           <xm:sqref>E53:E54</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{D8CAE4A4-473C-4F61-AE13-8FF934B8CBE5}">
+          <x14:cfRule type="cellIs" priority="61" operator="greaterThanOrEqual" id="{31DD1EDA-6559-4982-9E86-EF5D2479371C}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -3427,7 +3658,7 @@
           <xm:sqref>E53:E54</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{7C8897E3-6F1D-4499-AC0C-6F4C9CC2FBCF}">
+          <x14:cfRule type="cellIs" priority="62" operator="equal" id="{5C456A00-7193-4021-8CF8-FC73F0038748}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3438,7 +3669,7 @@
           <xm:sqref>E55</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{4B3F7461-A16D-4D3B-9D39-40FF32115ED0}">
+          <x14:cfRule type="cellIs" priority="63" operator="lessThanOrEqual" id="{07336C8A-B56C-4A92-A8A1-084AC9D101AD}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3455,7 +3686,7 @@
           <xm:sqref>E55</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{DEF384D9-8A22-49FC-AFEA-33DF8F4E0A59}">
+          <x14:cfRule type="cellIs" priority="64" operator="notBetween" id="{A66E47B6-8066-4342-9CF0-3A83FD0770D5}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -3473,7 +3704,7 @@
           <xm:sqref>E55</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{A7FD441F-0F85-41C0-A780-70717CB31913}">
+          <x14:cfRule type="cellIs" priority="65" operator="between" id="{EF4AA12E-8BBE-4079-8867-796DB009D152}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -3491,7 +3722,7 @@
           <xm:sqref>E55</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{15363016-1E5C-4EB6-8136-06F80ACC53AB}">
+          <x14:cfRule type="cellIs" priority="66" operator="greaterThanOrEqual" id="{6400EA18-21E5-4151-A753-85C1D5DCACCB}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -3508,7 +3739,7 @@
           <xm:sqref>E55</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{B8639A02-2B15-4A21-A66C-CD6625D77634}">
+          <x14:cfRule type="cellIs" priority="67" operator="equal" id="{E80F17E7-306C-4E0F-8A93-F8B07404A5E9}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3519,7 +3750,7 @@
           <xm:sqref>E56</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{3CC355C8-70A5-4D04-B513-21FC1588680E}">
+          <x14:cfRule type="cellIs" priority="68" operator="lessThanOrEqual" id="{6DBF1B98-937E-4418-B0ED-398B4B044384}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3536,7 +3767,7 @@
           <xm:sqref>E56</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{D6FA7885-FCF8-44EB-874E-2350E77735BD}">
+          <x14:cfRule type="cellIs" priority="69" operator="notBetween" id="{8089F7CA-D968-4F77-AF05-810248EF2EFC}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -3554,7 +3785,7 @@
           <xm:sqref>E56</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{838AE0F1-4674-4872-84C9-14406E44B8F6}">
+          <x14:cfRule type="cellIs" priority="70" operator="between" id="{DAEA66A7-584D-41AF-9470-819118F34D0E}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -3572,7 +3803,7 @@
           <xm:sqref>E56</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{F7CD0F60-2DFE-4B98-905E-6464719EF24C}">
+          <x14:cfRule type="cellIs" priority="71" operator="greaterThanOrEqual" id="{4C815E30-2934-4849-9AFC-EE93385E68ED}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -3589,7 +3820,7 @@
           <xm:sqref>E56</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{4E5DF751-BA4C-4721-8B13-4BE2F4378FF9}">
+          <x14:cfRule type="cellIs" priority="72" operator="equal" id="{1E007458-30D0-4FBA-8022-577DC1246203}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3600,7 +3831,7 @@
           <xm:sqref>E57:E58</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{20812B13-FB90-46BB-BBD2-6854F5FBBB89}">
+          <x14:cfRule type="cellIs" priority="73" operator="lessThanOrEqual" id="{962C396F-B826-40AF-B81F-D30A162E35BC}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3617,7 +3848,7 @@
           <xm:sqref>E57:E58</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{40B79EFF-4369-4C11-84C9-B6ABC130C926}">
+          <x14:cfRule type="cellIs" priority="74" operator="notBetween" id="{AFDDC927-09E3-46B4-8A3F-226D48E045F8}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -3635,7 +3866,7 @@
           <xm:sqref>E57:E58</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{DC7333BF-A919-44F6-98AB-0B531508152D}">
+          <x14:cfRule type="cellIs" priority="75" operator="between" id="{26164A4D-1A3B-4D3F-B4F8-9D20C30B6155}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -3653,7 +3884,7 @@
           <xm:sqref>E57:E58</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{FE1A2E6D-2A88-4FB1-8E68-ACBC7C1CBCAD}">
+          <x14:cfRule type="cellIs" priority="76" operator="greaterThanOrEqual" id="{E6601F6B-815A-4DB1-8BF1-7A95355F8F76}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -3670,7 +3901,7 @@
           <xm:sqref>E57:E58</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{C9467728-F633-4FE7-BA55-0B924C8032B6}">
+          <x14:cfRule type="cellIs" priority="77" operator="equal" id="{0CA5E311-9A76-4A2D-94F2-075136F6E4A6}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3681,7 +3912,7 @@
           <xm:sqref>E59</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{5662AB16-270E-4487-80F6-B7F6F2F7CC2F}">
+          <x14:cfRule type="cellIs" priority="78" operator="lessThanOrEqual" id="{96EAF195-E632-41CE-94EF-D75508FEBA4F}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -3698,7 +3929,7 @@
           <xm:sqref>E59</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{11F001CB-50E2-4F6E-91F9-7A6276E36E9E}">
+          <x14:cfRule type="cellIs" priority="79" operator="notBetween" id="{0E35AF53-1661-49BD-B850-A5F22F7D0491}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -3716,7 +3947,7 @@
           <xm:sqref>E59</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{ABEB53A4-8E24-4EDB-8317-CDB704CB279D}">
+          <x14:cfRule type="cellIs" priority="80" operator="between" id="{67C3C9EA-A713-4FD3-BD17-402D528A197F}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -3734,7 +3965,7 @@
           <xm:sqref>E59</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{68BBDC4C-2BFE-41AB-8895-434BB45CFBD8}">
+          <x14:cfRule type="cellIs" priority="81" operator="greaterThanOrEqual" id="{9F5A0A82-92C2-43F7-9903-CCB88612F7E8}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -3751,7 +3982,7 @@
           <xm:sqref>E59</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" text="Entregado" id="{4E00C9D4-9FFE-44CE-B53F-A0D13B2A43AB}">
+          <x14:cfRule type="containsText" priority="4" text="Entregado" id="{C040B42A-D759-447E-A515-18513431E93A}">
             <xm:f>NOT(ISERROR(SEARCH("Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3768,7 +3999,7 @@
           <xm:sqref>G13:G34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" text="No Entregado" id="{6F4D164F-1DF6-4C1F-8D7E-1013DFF67F3A}">
+          <x14:cfRule type="containsText" priority="3" text="No Entregado" id="{58AC9AD0-F09F-4B5A-833C-1B1D1CE80B60}">
             <xm:f>NOT(ISERROR(SEARCH("No Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3785,7 +4016,7 @@
           <xm:sqref>G13:G34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" text="En Desarrollo" id="{716A5B19-AEE5-4B47-B228-2B522AC9C334}">
+          <x14:cfRule type="containsText" priority="1" text="En Desarrollo" id="{8CD95E94-9937-4797-87F0-50DD37F6095C}">
             <xm:f>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3802,7 +4033,7 @@
           <xm:sqref>G13:G34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" text="Entregado" id="{D8312738-9E82-40A1-A415-CB762F3AA24B}">
+          <x14:cfRule type="containsText" priority="82" text="Entregado" id="{67DC19FF-D526-4914-84AE-83BF6E7BC1DB}">
             <xm:f>NOT(ISERROR(SEARCH("Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3819,7 +4050,7 @@
           <xm:sqref>G36:G39</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" text="No Entregado" id="{D4AC4497-CB0E-4ECB-A75A-CFAEB349DCA2}">
+          <x14:cfRule type="containsText" priority="83" text="No Entregado" id="{CE37F5C8-AC93-4CC9-800F-1A842510B76B}">
             <xm:f>NOT(ISERROR(SEARCH("No Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3836,7 +4067,7 @@
           <xm:sqref>G36:G39</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" text="En Desarrollo" id="{8EA16F93-2C7C-40C6-9A95-000A53FA4B5D}">
+          <x14:cfRule type="containsText" priority="84" text="En Desarrollo" id="{56FCC69D-E718-41AB-9E46-45D3E73A48E8}">
             <xm:f>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3853,7 +4084,7 @@
           <xm:sqref>G36:G39</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" text="Entregado" id="{D98E7D2C-6296-410E-AB47-353AAD2E9BBD}">
+          <x14:cfRule type="containsText" priority="85" text="Entregado" id="{9A28AB3D-7287-49DE-B1F4-C93C33F3E33F}">
             <xm:f>NOT(ISERROR(SEARCH("Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3870,7 +4101,7 @@
           <xm:sqref>G40:G42</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" text="No Entregado" id="{46A02842-057E-4165-BB25-5D8A699750FC}">
+          <x14:cfRule type="containsText" priority="86" text="No Entregado" id="{53E377BD-428A-487B-8821-9C5D1B84BC46}">
             <xm:f>NOT(ISERROR(SEARCH("No Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3887,7 +4118,7 @@
           <xm:sqref>G40:G42</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" text="En Desarrollo" id="{5F9F2C1F-9167-4147-8640-850A7E59483E}">
+          <x14:cfRule type="containsText" priority="87" text="En Desarrollo" id="{44EE2C73-163A-4681-9689-BC63B4FAEDC1}">
             <xm:f>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3904,7 +4135,7 @@
           <xm:sqref>G40:G42</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" text="Entregado" id="{ECC072AF-5F39-4013-9C3F-B9CEF549900B}">
+          <x14:cfRule type="containsText" priority="88" text="Entregado" id="{095B6997-CD2F-440E-AABF-85C590CD888E}">
             <xm:f>NOT(ISERROR(SEARCH("Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3921,7 +4152,7 @@
           <xm:sqref>G43:G45</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" text="No Entregado" id="{D463EF46-6419-4C28-9840-D3FD157DF986}">
+          <x14:cfRule type="containsText" priority="89" text="No Entregado" id="{2A3D1DDD-6BB7-4C7D-B710-3FD37704ADE1}">
             <xm:f>NOT(ISERROR(SEARCH("No Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3938,7 +4169,7 @@
           <xm:sqref>G43:G45</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" text="En Desarrollo" id="{9193EA16-11CC-4894-9253-288831C43498}">
+          <x14:cfRule type="containsText" priority="90" text="En Desarrollo" id="{869393F2-E0AF-436D-B64F-C7BED6DF413D}">
             <xm:f>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3955,7 +4186,7 @@
           <xm:sqref>G43:G45</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" text="Entregado" id="{D6C76DF9-FB5C-4436-85ED-E45D29C9396E}">
+          <x14:cfRule type="containsText" priority="91" text="Entregado" id="{64CEC4DF-F0AA-4D97-8F78-14C67F5BD9B9}">
             <xm:f>NOT(ISERROR(SEARCH("Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3972,7 +4203,7 @@
           <xm:sqref>G46:G48</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" text="No Entregado" id="{DF1E8574-5988-47E3-9AF3-B87C5CF6997C}">
+          <x14:cfRule type="containsText" priority="92" text="No Entregado" id="{3BA9353B-7869-49D6-BE66-D0D6ABC5EB86}">
             <xm:f>NOT(ISERROR(SEARCH("No Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -3989,7 +4220,7 @@
           <xm:sqref>G46:G48</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" text="En Desarrollo" id="{686B0FB6-38DD-4072-A9E7-4323215A885E}">
+          <x14:cfRule type="containsText" priority="93" text="En Desarrollo" id="{3942900B-8FEE-4983-9B4E-91C8021E4ECE}">
             <xm:f>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4006,7 +4237,7 @@
           <xm:sqref>G46:G48</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" text="Entregado" id="{0F8E0B1B-A335-47BE-A8CC-435BC0C30A50}">
+          <x14:cfRule type="containsText" priority="94" text="Entregado" id="{B64B3D7E-1148-4DCB-9E02-101F9ED49C42}">
             <xm:f>NOT(ISERROR(SEARCH("Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4023,7 +4254,7 @@
           <xm:sqref>G49:G51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" text="No Entregado" id="{518E7CA8-56BD-4AA2-A5D6-1463BFA0750F}">
+          <x14:cfRule type="containsText" priority="95" text="No Entregado" id="{EA9A40A3-8C73-4683-9882-9F8E22F1BD9B}">
             <xm:f>NOT(ISERROR(SEARCH("No Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4040,7 +4271,7 @@
           <xm:sqref>G49:G51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" text="En Desarrollo" id="{BDC4E650-64C3-475A-9895-D4ED962C7773}">
+          <x14:cfRule type="containsText" priority="96" text="En Desarrollo" id="{FBFF8F1F-D7CB-4616-9474-6EF93475A031}">
             <xm:f>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4057,7 +4288,7 @@
           <xm:sqref>G49:G51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" text="Entregado" id="{DAF91B78-E84C-4162-8E99-60C9A2B13B59}">
+          <x14:cfRule type="containsText" priority="97" text="Entregado" id="{DAF1FD18-42B8-4546-AAEA-382B7CDDBC77}">
             <xm:f>NOT(ISERROR(SEARCH("Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4074,7 +4305,7 @@
           <xm:sqref>G52:G54</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" text="No Entregado" id="{A168FF30-E5DC-47FD-B996-F838E50D82FD}">
+          <x14:cfRule type="containsText" priority="98" text="No Entregado" id="{140E5DD6-989E-4A41-8774-A108F63A91E5}">
             <xm:f>NOT(ISERROR(SEARCH("No Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4091,7 +4322,7 @@
           <xm:sqref>G52:G54</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" text="En Desarrollo" id="{F079A5CC-0227-4FD3-8AFE-AA42E3F134FB}">
+          <x14:cfRule type="containsText" priority="99" text="En Desarrollo" id="{8216BFA2-4981-4AAB-A752-A9C3256456FB}">
             <xm:f>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4108,7 +4339,7 @@
           <xm:sqref>G52:G54</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" text="Entregado" id="{DA142265-458A-4E09-ABBF-545EA6267E38}">
+          <x14:cfRule type="containsText" priority="100" text="Entregado" id="{9AF1D934-FEB4-454C-8300-2052C50ADF70}">
             <xm:f>NOT(ISERROR(SEARCH("Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4125,7 +4356,7 @@
           <xm:sqref>G55:G57</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" text="No Entregado" id="{25CCE73C-045A-4483-9279-E286426DDDA9}">
+          <x14:cfRule type="containsText" priority="101" text="No Entregado" id="{36E6F605-3FCE-43A0-90E5-7554AA93EE31}">
             <xm:f>NOT(ISERROR(SEARCH("No Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4142,7 +4373,7 @@
           <xm:sqref>G55:G57</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" text="En Desarrollo" id="{684ACBF6-E26C-410F-8E5A-0284BC7A9689}">
+          <x14:cfRule type="containsText" priority="102" text="En Desarrollo" id="{268B07B2-0286-48B5-96CD-B817480C6F5D}">
             <xm:f>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4159,7 +4390,7 @@
           <xm:sqref>G55:G57</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" text="Entregado" id="{70F21F55-CDC3-46C9-9132-213CD27220FA}">
+          <x14:cfRule type="containsText" priority="103" text="Entregado" id="{1C4C45AD-CDD7-4C52-A671-41B37CA73137}">
             <xm:f>NOT(ISERROR(SEARCH("Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4176,7 +4407,7 @@
           <xm:sqref>G58:G59</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" text="No Entregado" id="{15EE6AA6-A024-4CCC-A3D6-EAD70261293A}">
+          <x14:cfRule type="containsText" priority="104" text="No Entregado" id="{A7A4F19B-9707-425E-A6D8-8A1BE82FD904}">
             <xm:f>NOT(ISERROR(SEARCH("No Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4193,7 +4424,7 @@
           <xm:sqref>G58:G59</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" text="En Desarrollo" id="{6AA4819B-A7C2-4E4E-8DC8-EE96A336A831}">
+          <x14:cfRule type="containsText" priority="105" text="En Desarrollo" id="{54BA8557-A234-4EF7-874C-2EC2A901B676}">
             <xm:f>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4210,7 +4441,7 @@
           <xm:sqref>G58:G59</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{9A2A70DD-F0A3-41D6-80E4-27FAE92EFB92}">
+          <x14:cfRule type="cellIs" priority="106" operator="equal" id="{05AEB4B4-0FBB-4346-A13B-F5BBFFFA24C8}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -4221,7 +4452,7 @@
           <xm:sqref>E61:E69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="lessThanOrEqual" id="{E3777069-0F6C-49DC-A0BE-526E4EE350C3}">
+          <x14:cfRule type="cellIs" priority="107" operator="lessThanOrEqual" id="{B8AA18FF-616B-4C8A-A2ED-855227E5FDDB}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -4238,7 +4469,7 @@
           <xm:sqref>E61:E69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="notBetween" id="{532C5D50-D9DF-4D92-B0A9-4EF6C98B1058}">
+          <x14:cfRule type="cellIs" priority="108" operator="notBetween" id="{42E4B005-02E3-4A68-AEC9-DAEBCA31BBE8}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -4256,7 +4487,7 @@
           <xm:sqref>E61:E69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="between" id="{706E98ED-52BA-4ADD-BCE9-5EA0F1BEF763}">
+          <x14:cfRule type="cellIs" priority="109" operator="between" id="{4BFB7CBA-8DD3-4612-B5E9-CE6F520A334A}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -4274,7 +4505,7 @@
           <xm:sqref>E61:E69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{B1777056-97B2-482B-8608-8718AEF2EB90}">
+          <x14:cfRule type="cellIs" priority="110" operator="greaterThanOrEqual" id="{7C148D47-3F97-41DD-896D-A1B9C0DE8E55}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -4291,7 +4522,7 @@
           <xm:sqref>E61:E69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" text="Entregado" id="{A33FDF71-97F4-437F-9208-03EA0398C629}">
+          <x14:cfRule type="containsText" priority="111" text="Entregado" id="{A39065B9-8A75-4B16-AD5B-6F0786037521}">
             <xm:f>NOT(ISERROR(SEARCH("Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4308,7 +4539,7 @@
           <xm:sqref>G61:G69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" text="No Entregado" id="{B16DC2F5-F673-42F4-8A33-13EC5B47DBE1}">
+          <x14:cfRule type="containsText" priority="112" text="No Entregado" id="{6EDBC02F-F735-4742-A930-67A444C73C1F}">
             <xm:f>NOT(ISERROR(SEARCH("No Entregado",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4325,7 +4556,7 @@
           <xm:sqref>G61:G69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" text="En Desarrollo" id="{742010CC-CF1F-41D2-90B3-1DDD47A34334}">
+          <x14:cfRule type="containsText" priority="113" text="En Desarrollo" id="{BBFC9594-AD77-4AD8-9430-DF444CD02EF7}">
             <xm:f>NOT(ISERROR(SEARCH("En Desarrollo",G13)))</xm:f>
             <x14:dxf>
               <font>
@@ -4345,121 +4576,121 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="20" disablePrompts="0">
-        <x14:dataValidation xr:uid="{5AC8AFF1-379C-48C1-8415-D29E35367D10}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{48B851AC-5A2C-4D34-87B3-0330F52B812E}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$B$4:$B$8</xm:f>
           </x14:formula1>
           <xm:sqref>F13:F34</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{04D5338D-24BC-4A69-BA7A-50913B0ECF3F}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{2F284D9E-8633-4D6B-9E4F-04F4A6BDCC1E}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$F$4:$F$6</xm:f>
           </x14:formula1>
           <xm:sqref>G13:G34</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{392350BA-71D8-4131-8FA0-972B3DB3F3B4}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{A7C7734B-E4A7-4BF2-BE1F-6F49C877725C}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$F$4:$F$6</xm:f>
           </x14:formula1>
           <xm:sqref>G36:G39</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{F40DFCA9-D4B1-4AD4-93FD-DDAC130CCBC6}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{4B6AAD6F-256C-4618-A117-662F7CFB8B39}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$F$4:$F$6</xm:f>
           </x14:formula1>
           <xm:sqref>G40:G42</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{0F281E81-1A2D-4E00-ACE8-01F001B75888}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{44E14E6A-696E-48DA-9C59-67CF87F53AEF}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$F$4:$F$6</xm:f>
           </x14:formula1>
           <xm:sqref>G43:G45</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{6066F420-118E-4D17-A7A8-404559BB4147}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{3C74AEF3-B59A-4135-995D-084BEC34195D}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$F$4:$F$6</xm:f>
           </x14:formula1>
           <xm:sqref>G46:G48</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{12534331-4641-4FD1-A877-F3567A90116E}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{C391DC4D-E774-468A-ADF3-F2D8B3B588F5}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$F$4:$F$6</xm:f>
           </x14:formula1>
           <xm:sqref>G49:G51</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{78076B26-50EB-430E-A397-223E2BF810DC}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{D11C97F8-53A4-44D4-AEA7-C2681177136F}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$F$4:$F$6</xm:f>
           </x14:formula1>
           <xm:sqref>G52:G54</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{A1E21F89-369A-4DA2-8847-45E745DD3F97}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{F9714950-9865-496F-8DBA-32BB1388234B}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$F$4:$F$6</xm:f>
           </x14:formula1>
           <xm:sqref>G55:G57</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{DE965A2B-7838-429C-91DD-881B627D9134}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{720B718A-AFF6-454B-ABFE-7D64B3BDB71E}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$F$4:$F$6</xm:f>
           </x14:formula1>
           <xm:sqref>G58:G59</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{F185D83B-5740-4866-9197-1B447C6B5352}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{ACA4F691-526E-459B-86FA-4FD18171EDFB}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$B$4:$B$8</xm:f>
           </x14:formula1>
           <xm:sqref>F36:F39</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{9140D37E-6BB1-48BC-9A7A-89E3CDA35F0E}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{46145344-2806-4A6D-B270-867D748D7974}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$B$4:$B$8</xm:f>
           </x14:formula1>
           <xm:sqref>F40:F42</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{FA54E6B2-774B-4878-9595-156E1C5905EC}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{DB4ADE88-2AE6-460C-A27B-DA14964C0927}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$B$4:$B$8</xm:f>
           </x14:formula1>
           <xm:sqref>F43:F45</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{298FED5C-404B-46FC-8111-AF988B9D309D}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{54917AFF-7903-4197-A4BD-691856D8D967}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$B$4:$B$8</xm:f>
           </x14:formula1>
           <xm:sqref>F46:F48</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{85D4E9E2-878E-4C73-8D7D-B7178E515056}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{31780CE1-4766-4DE7-B587-07D9016D2AE6}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$B$4:$B$8</xm:f>
           </x14:formula1>
           <xm:sqref>F49:F51</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{EC3BCD86-F6E8-4147-9406-E9088C4D2B9F}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{353F2E4A-F77D-4B0E-8DC1-DDCCF3E82BD8}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$B$4:$B$8</xm:f>
           </x14:formula1>
           <xm:sqref>F52:F54</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{86DD180B-98A7-4FAC-9306-930C00307805}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{F7BDAF66-D709-4898-A8D9-EB8DE143C31C}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$B$4:$B$8</xm:f>
           </x14:formula1>
           <xm:sqref>F55:F57</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{73A60588-16C9-4D02-ABF8-51DA8CD1EAF8}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{7586BF43-5059-4F26-82BA-6F32FBC52809}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$B$4:$B$8</xm:f>
           </x14:formula1>
           <xm:sqref>F58:F59</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{E446303C-8441-42F1-8612-104AB291081F}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{9352F272-F241-4AB0-B318-015F5AB1D963}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$F$4:$F$6</xm:f>
           </x14:formula1>
           <xm:sqref>G61 G62 G63 G64 G65 G66 G67 G68 G69</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{C8BD5A57-C518-4786-9EA5-067D0D34C8A9}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{A1A5AD1D-804B-4540-9779-E7F257365B90}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$B$4:$B$8</xm:f>
           </x14:formula1>

</xml_diff>